<commit_message>
GCC Landscape: re-judge flags under clarified definitions
Insurance Operations = all core insurance functions; Finance includes
financial reporting and local finance leadership. Duplicate entity rows
aligned; legend updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0122CtMb1m8jYJ2C8cYtjtCe
</commit_message>
<xml_diff>
--- a/GCC_Landscape_Oct26.xlsx
+++ b/GCC_Landscape_Oct26.xlsx
@@ -2091,7 +2091,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="119.85" customHeight="1">
+    <row r="11" ht="181.95" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
           <r>
@@ -2140,19 +2140,19 @@
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I11" s="14" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H11" s="14" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I11" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="J11" s="15" t="inlineStr">
         <is>
           <r>
@@ -2179,6 +2179,22 @@
               <sz val="9"/>
             </rPr>
             <t>Shift to output-based model built on technology, automation and AI (Feb 2025): application development, data analytics, AI; 160k sq ft Pune expansion Oct 2024.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">
+Finance: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Corporate-function operations including finance are a stated Centre of Excellence domain delivered from Bengaluru and Pune for 35+ AXA entities in 14 countries (Feb 2025).</t>
           </r>
           <r>
             <rPr>
@@ -2218,6 +2234,26 @@
             <t xml:space="preserve">
 https://www.business-standard.com/content/press-releases-ani/axa-global-business-services-embarks-on-a-new-era-of-transformation-as-it-celebrates-30-years-in-india-125021300860_1.html
 https://www.prnewswire.com/in/news-releases/axa-unveils-state-of-the-art-office-space-in-pune-expands-its-global-business-services-center-302271407.html</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+Finance:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF0563C1"/>
+              <sz val="8"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+https://www.tribuneindia.com/news/business/axa-global-business-services-embarks-on-a-new-era-of-transformation-as-it-celebrates-30-years-in-india/
+https://tracxn.com/d/legal-entities/india/axa-global-business-services-private-limited/__YU7KMI_cCEU4d_R8dX_1H3gmvZ32z1HhrCxNpWhXrV0</t>
           </r>
           <r>
             <rPr>
@@ -4922,7 +4958,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="54.3" customHeight="1">
+    <row r="23" ht="75" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
           <r>
@@ -4971,19 +5007,19 @@
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H23" s="14" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H23" s="14" t="inlineStr">
+      <c r="I23" s="14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I23" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="J23" s="15" t="inlineStr">
         <is>
           <r>
@@ -5010,6 +5046,22 @@
               <sz val="9"/>
             </rPr>
             <t>Global Business Solutions runs groupwide capability hubs in Bengaluru and Hyderabad, with Hyderabad positioned as the analytical and innovation hub for digital, data and technology (2026).</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">
+Finance: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Group Finance work runs from Bengaluru: ~70-strong Subledger Liabilities team owns L&amp;H and P&amp;C sub-ledger accounting under US GAAP, STAT and IFRS, plus finance-operations and AI/automation roles (2025-26).</t>
           </r>
           <r>
             <rPr>
@@ -5043,6 +5095,25 @@
             <t xml:space="preserve">
 https://www.swissre.com/profile/Amit_Kalra/ip_f2cb75</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+Finance:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF0563C1"/>
+              <sz val="8"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+https://careers.swissre.com/job/Bangalore-Accountant-II-KA/1199902701</t>
+          </r>
         </is>
       </c>
       <c r="L23" s="15" t="inlineStr">
@@ -5117,7 +5188,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="109.5" customHeight="1">
+    <row r="24" ht="181.95" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
           <r>
@@ -5166,19 +5237,19 @@
       </c>
       <c r="G24" s="18" t="inlineStr">
         <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H24" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I24" s="18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="J24" s="19" t="inlineStr">
         <is>
           <r>
@@ -5205,6 +5276,22 @@
               <sz val="9"/>
             </rPr>
             <t>Permanent Bengaluru GCC inaugurated Apr 2026 for AI engineering, cloud platforms, data and analytics; in-housing vendor technology work, headcount doubling to ~400 by end-2026.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">
+Finance: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Local finance leadership being built out at the Bengaluru and Pune sites (Aug 2026), with Country Head Mohua Sengupta overseeing financial, regulatory and compliance matters since Nov 2025.</t>
           </r>
           <r>
             <rPr>
@@ -5254,6 +5341,26 @@
             <t xml:space="preserve">
 https://www.peoplematters.in/news/business/the-standard-grows-india-gcc-to-400-positioning-bengaluru-at-the-centre-of-its-innovation-strategy-51594
 https://www.thepeoplesboard.com/?p=17616</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+Finance:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF0563C1"/>
+              <sz val="8"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+https://www.peoplematters.in/news/business/the-standard-grows-india-gcc-to-400-positioning-bengaluru-at-the-centre-of-its-innovation-strategy-51594
+https://gcc.economictimes.indiatimes.com/news/the-standard-expands-global-footprint-with-new-office-and-mohua-sengupta-as-country-head-in-india/125379556</t>
           </r>
           <r>
             <rPr>
@@ -8106,7 +8213,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="99.14999999999999" customHeight="1">
+    <row r="36" ht="119.85" customHeight="1">
       <c r="A36" s="16" t="inlineStr">
         <is>
           <r>
@@ -8155,19 +8262,19 @@
       </c>
       <c r="G36" s="18" t="inlineStr">
         <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H36" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I36" s="18" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H36" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I36" s="18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="J36" s="19" t="inlineStr">
         <is>
           <r>
@@ -8194,6 +8301,22 @@
               <sz val="9"/>
             </rPr>
             <t>Hyderabad GCC launched Apr 2026 with 1,000+ roles across cloud engineering, data and AI, application development, cybersecurity and quality engineering; Amit Kalra heads it from Jul 2026.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">
+Finance: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Site-level finance, procurement and vendor governance set up under new GCC COO Ganesh Rao (mid-2026), formerly Principal Financial's Head of Shared Services.</t>
           </r>
           <r>
             <rPr>
@@ -8243,6 +8366,25 @@
             <t xml:space="preserve">
 https://reinsurancene.ws/zurich-appoints-amit-kalra-to-lead-new-global-capability-center-in-india/
 https://explorer.hub71.com/news/feed/zurich-insurance-launches-global-capability-center-in-hyderabad-to-advance-ai-and-tech-capabilities</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+Finance:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF0563C1"/>
+              <sz val="8"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+https://www.cxodigitalpulse.com/?p=61973</t>
           </r>
           <r>
             <rPr>
@@ -9688,7 +9830,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="140.55" customHeight="1">
+    <row r="43" ht="192.3" customHeight="1">
       <c r="A43" s="12" t="inlineStr">
         <is>
           <r>
@@ -9737,7 +9879,7 @@
       </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="H43" s="14" t="inlineStr">
@@ -9776,6 +9918,22 @@
               <sz val="9"/>
             </rPr>
             <t>Second GCC opened in Hyderabad Jun 2026 taking India past 3,000 staff: technology, engineering, automation, analytics and GenAI application development for Health, Wealth and Investment Management.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">
+Finance: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t>SOX and finance-controls team in Bengaluru (2026 hiring) supports Finance and Accounting on control documentation, testing and remediation, extending financial-reporting controls work to India.</t>
           </r>
           <r>
             <rPr>
@@ -9831,6 +9989,26 @@
             <t xml:space="preserve">
 https://gcc.economictimes.indiatimes.com/news/workplace-transformation/voya-financial-expands-presence-with-new-global-capability-center-in-hyderabad/131633042
 https://www.instahyre.com/job-332378-gen-ai-app-developer-at-voya-india-bangalore/</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+Finance:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF0563C1"/>
+              <sz val="8"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+https://accajobs.quintedge.com/jobs/sox-compliance-analyst-voya-india-7qbke6
+https://joinsaarthi.com/jobs/voya-financial/senior-associate-36367-bengaluru/5d4252df-6baa-49ac-89c2-13d092fefa5e</t>
           </r>
           <r>
             <rPr>
@@ -10194,7 +10372,7 @@
       <c r="K45" s="10" t="n"/>
       <c r="L45" s="11" t="n"/>
     </row>
-    <row r="46" ht="57.75" customHeight="1">
+    <row r="46" ht="78.45" customHeight="1">
       <c r="A46" s="12" t="inlineStr">
         <is>
           <r>
@@ -10243,19 +10421,19 @@
       </c>
       <c r="G46" s="14" t="inlineStr">
         <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H46" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I46" s="14" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H46" s="14" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I46" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="J46" s="15" t="inlineStr">
         <is>
           <r>
@@ -10266,6 +10444,22 @@
               <sz val="9"/>
             </rPr>
             <t>Facultative reinsurance underwriting branch (Mumbai)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">
+Finance: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Local CFO Avneet Kumar Gupta sits among the Mumbai branch's key managerial persons alongside CEO and CUO, giving branch-level finance and statutory reporting capability (2025-26).</t>
           </r>
           <r>
             <rPr>
@@ -10303,7 +10497,26 @@
               <b val="1"/>
               <sz val="8"/>
             </rPr>
-            <t>Insurance Operations:</t>
+            <t>Finance:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF0563C1"/>
+              <sz val="8"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+https://axaxl.com/reinsurance/our-companies/xl-insurance-company-se</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+Insurance Operations:</t>
           </r>
           <r>
             <rPr>
@@ -12095,7 +12308,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="54.3" customHeight="1">
+    <row r="55" ht="75" customHeight="1">
       <c r="A55" s="16" t="inlineStr">
         <is>
           <r>
@@ -12144,19 +12357,19 @@
       </c>
       <c r="G55" s="18" t="inlineStr">
         <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H55" s="18" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I55" s="18" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H55" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I55" s="18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="J55" s="19" t="inlineStr">
         <is>
           <r>
@@ -12167,6 +12380,22 @@
               <sz val="9"/>
             </rPr>
             <t>Facultative reinsurance underwriting branch (Mumbai)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">
+Finance: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Local CFO Avneet Kumar Gupta sits among the Mumbai branch's key managerial persons alongside CEO and CUO, giving branch-level finance and statutory reporting capability (2025-26).</t>
           </r>
           <r>
             <rPr>
@@ -12204,7 +12433,26 @@
               <b val="1"/>
               <sz val="8"/>
             </rPr>
-            <t>Insurance Operations:</t>
+            <t>Finance:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF0563C1"/>
+              <sz val="8"/>
+              <u val="single"/>
+            </rPr>
+            <t xml:space="preserve">
+https://axaxl.com/reinsurance/our-companies/xl-insurance-company-se</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+Insurance Operations:</t>
           </r>
           <r>
             <rPr>
@@ -13473,7 +13721,7 @@
               <rFont val="Arial"/>
               <sz val="9"/>
             </rPr>
-            <t>In-branch finance and administration lead appointed Aug 2026 (ex-GIC Re): accounting, taxation, regulatory reporting and credit control for the GIFT City branch.</t>
+            <t>In-branch finance and administration lead appointed Aug 2026 (ex-GIC Re): finance, taxation, regulatory compliance, audit management and credit control for the GIFT City branch.</t>
           </r>
           <r>
             <rPr>
@@ -13489,7 +13737,7 @@
               <rFont val="Arial"/>
               <sz val="9"/>
             </rPr>
-            <t>IFSCA branch approved Feb 2026; Head of India Chaturbhuj Bansal from Jun 2026 building a non-life treaty underwriting team, senior treaty underwriter hired Aug 2026.</t>
+            <t>IFSCA branch approved Feb 2026; Head of India Chaturbhuj Bansal (Jun 2026) building a non-life treaty underwriting and cat-modelling team, senior treaty underwriter hired Aug 2026.</t>
           </r>
           <r>
             <rPr>
@@ -14131,7 +14379,7 @@
               <rFont val="Arial"/>
               <sz val="9"/>
             </rPr>
-            <t>GIFT City branch approved Feb 2026 as PartnerRe's first India presence; CEO India Ankur Gupta from Jun 2026 serving Indian cedants with local P&amp;C underwriting.</t>
+            <t>GIFT City branch approved Feb 2026 as PartnerRe's first India presence; CEO India Ankur Gupta from Jun 2026 serving Indian cedants locally with P&amp;C reinsurance underwriting.</t>
           </r>
           <r>
             <rPr>
@@ -16643,10 +16891,10 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="40" customHeight="1">
+    <row r="79" ht="64" customHeight="1">
       <c r="A79" s="20" t="inlineStr">
         <is>
-          <t>Legend: a tick in Technology / Finance / Insurance Operations / Internal Audit (SOX, ICFR) means verified evidence that the function is performed or being built in India within roughly the past 1-2 years; the focus column states why each flagged bucket is flagged and the underlying trend; the source column lists the links per bucket; the last column reconciles the team's original entries per bucket (kept / dropped with reason / newly added). Group-level or parent news, registry revenue figures and bare licence events do not earn a tick. Evidence base: Oct 2026 research and audit of columns O-R (see Focus Review Log).</t>
+          <t>Legend: a tick means verified evidence that the function is performed or being built in India within roughly the past 1-2 years. Technology = engineering, software, AI/GenAI, data, cloud, cybersecurity, digital platforms, automation. Finance = finance and accounting incl. financial reporting (statutory/regulatory, IFRS/US GAAP), sub-ledger and technical accounting, close, FP&amp;A, treasury, tax, procurement, local CFO/finance lead. Insurance Ops = all core insurance functions: underwriting and pricing, actuarial, claims, policy administration, reinsurance (treaty/facultative, lines written, licence), product, distribution/broking support, customer service, insurance analytics. Internal Audit = SOX/ICFR testing, internal audit, controls assurance. The focus column states why each flagged bucket is flagged and the trend; the source column lists links per bucket; the last column reconciles the team's original entries per bucket (kept / dropped with reason / newly added). Group-level or parent news, registry revenue figures and bare licence events do not earn a tick. Evidence base: Oct 2026 research and audit of columns O-R (see Focus Review Log).</t>
         </is>
       </c>
     </row>

</xml_diff>